<commit_message>
[BOÎTE À OUTILS] Nettoie le modèle d'annuaire de crise
</commit_message>
<xml_diff>
--- a/back/src/api/outils/modele-annuaire-de-crise.xlsx
+++ b/back/src/api/outils/modele-annuaire-de-crise.xlsx
@@ -1,52 +1,57 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Version du XXXX202X" sheetId="1" r:id="rId5"/>
+    <sheet name="Version du XXXX202X" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <r>
       <rPr>
+        <b val="false"/>
+        <sz val="22"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b val="0"/>
-        <color theme="1"/>
-        <sz val="22.0"/>
       </rPr>
-      <t>Template de liste de contacts à télécharger</t>
+      <t xml:space="preserve">Template de liste de contacts à télécharger</t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="22"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="22.0"/>
       </rPr>
       <t xml:space="preserve">
 </t>
     </r>
     <r>
       <rPr>
+        <b val="false"/>
+        <color rgb="FF666666"/>
         <rFont val="Arial"/>
-        <b val="0"/>
-        <color rgb="FF666666"/>
       </rPr>
-      <t>Ce fichier vous est fourni par MesServicesCyber</t>
+      <t xml:space="preserve">Ce fichier vous est fourni par MesServicesCyber</t>
     </r>
   </si>
   <si>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t xml:space="preserve">Voici les bonnes pratiques de mise à jour de ce fichier :
 1 - Désigner un responsable de la mise à jour de cette liste d'outils.
@@ -57,21 +62,21 @@
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color indexed="2"/>
         <rFont val="Arial"/>
-        <color rgb="FFFF0000"/>
-        <sz val="11.0"/>
       </rPr>
       <t xml:space="preserve">Information obligatoire*
 </t>
     </r>
     <r>
       <rPr>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <i/>
-        <color theme="1"/>
-        <sz val="9.0"/>
       </rPr>
-      <t>Une ligne d'exemple est fourni pour remplir ce document ci-dessous :</t>
+      <t xml:space="preserve">Une ligne d'exemple est fourni pour remplir ce document ci-dessous :</t>
     </r>
   </si>
   <si>
@@ -80,17 +85,17 @@
   <si>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
-      <t>Nom prénom</t>
+      <t xml:space="preserve">Nom prénom</t>
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color indexed="2"/>
         <rFont val="Arial"/>
-        <color rgb="FFFF0000"/>
-        <sz val="11.0"/>
       </rPr>
       <t>*</t>
     </r>
@@ -98,17 +103,17 @@
   <si>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t>Fonction</t>
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color indexed="2"/>
         <rFont val="Arial"/>
-        <color rgb="FFFF0000"/>
-        <sz val="11.0"/>
       </rPr>
       <t>*</t>
     </r>
@@ -116,17 +121,17 @@
   <si>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t>Téléphone</t>
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color indexed="2"/>
         <rFont val="Arial"/>
-        <color rgb="FFFF0000"/>
-        <sz val="11.0"/>
       </rPr>
       <t>*</t>
     </r>
@@ -134,41 +139,41 @@
   <si>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t>Email</t>
     </r>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color indexed="2"/>
         <rFont val="Arial"/>
-        <color rgb="FFFF0000"/>
-        <sz val="11.0"/>
       </rPr>
       <t>*</t>
     </r>
   </si>
   <si>
-    <t>Email de secours</t>
+    <t xml:space="preserve">Email de secours</t>
   </si>
   <si>
     <t>Statut</t>
   </si>
   <si>
-    <t>Données complémentaires</t>
+    <t xml:space="preserve">Données complémentaires</t>
   </si>
   <si>
-    <t>IT / prestataire infogérant</t>
+    <t xml:space="preserve">IT / prestataire infogérant</t>
   </si>
   <si>
-    <t>Aline Dupont</t>
+    <t xml:space="preserve">Aline Dupont</t>
   </si>
   <si>
-    <t>Responsable projet</t>
+    <t xml:space="preserve">Responsable projet</t>
   </si>
   <si>
-    <t>01 02 03 04 05</t>
+    <t xml:space="preserve">01 02 03 04 05</t>
   </si>
   <si>
     <t>alinee.dupont@exemple.fr</t>
@@ -188,10 +193,10 @@
     <t xml:space="preserve">Pierre Kermarrec (suppléant d'Aline) </t>
   </si>
   <si>
-    <t>Adjoint Responsable projet</t>
+    <t xml:space="preserve">Adjoint Responsable projet</t>
   </si>
   <si>
-    <t>01 03 02 04 05</t>
+    <t xml:space="preserve">01 03 02 04 05</t>
   </si>
   <si>
     <t>pierre.kermarrec@exemple.fr</t>
@@ -202,19 +207,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
-      <t>Nom prénom</t>
+      <t xml:space="preserve">Nom prénom</t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color indexed="2"/>
         <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFFF0000"/>
-        <sz val="11.0"/>
       </rPr>
       <t>*</t>
     </r>
@@ -222,19 +227,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t>Fonction</t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color indexed="2"/>
         <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFFF0000"/>
-        <sz val="11.0"/>
       </rPr>
       <t>*</t>
     </r>
@@ -242,19 +247,19 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t>Téléphone</t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color indexed="2"/>
         <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFFF0000"/>
-        <sz val="11.0"/>
       </rPr>
       <t>*</t>
     </r>
@@ -262,25 +267,25 @@
   <si>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <b/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t>Email</t>
     </r>
     <r>
       <rPr>
+        <b/>
+        <sz val="11"/>
+        <color indexed="2"/>
         <rFont val="Arial"/>
-        <b/>
-        <color rgb="FFFF0000"/>
-        <sz val="11.0"/>
       </rPr>
       <t>*</t>
     </r>
   </si>
   <si>
-    <t>Décideur / dirigeant</t>
+    <t xml:space="preserve">Décideur / dirigeant</t>
   </si>
   <si>
     <t>RSSI</t>
@@ -307,10 +312,10 @@
     <t>Logistique</t>
   </si>
   <si>
-    <t>Référent PCA/PRA</t>
+    <t xml:space="preserve">Référent PCA/PRA</t>
   </si>
   <si>
-    <t>Responsable métier</t>
+    <t xml:space="preserve">Responsable métier</t>
   </si>
   <si>
     <t>SOC</t>
@@ -328,21 +333,21 @@
 - numéro de compte : </t>
   </si>
   <si>
-    <t>Autres fournisseurs critiques</t>
+    <t xml:space="preserve">Autres fournisseurs critiques</t>
   </si>
   <si>
-    <t>Prestataires de sauvegardes 
+    <t xml:space="preserve">Prestataires de sauvegardes 
 (si différents)</t>
   </si>
   <si>
-    <t>Assureur cyber</t>
+    <t xml:space="preserve">Assureur cyber</t>
   </si>
   <si>
-    <t>Conditionnel 
+    <t xml:space="preserve">Conditionnel 
 (si souscrit)</t>
   </si>
   <si>
-    <t>Opérateur télécom</t>
+    <t xml:space="preserve">Opérateur télécom</t>
   </si>
   <si>
     <t>Banque</t>
@@ -351,10 +356,10 @@
     <t xml:space="preserve">Contacts régionaux </t>
   </si>
   <si>
-    <t>Contacts sectoriels</t>
+    <t xml:space="preserve">Contacts sectoriels</t>
   </si>
   <si>
-    <t>Contacts nationaux</t>
+    <t xml:space="preserve">Contacts nationaux</t>
   </si>
   <si>
     <t>CNIL</t>
@@ -362,35 +367,35 @@
   <si>
     <r>
       <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
         <rFont val="Arial"/>
-        <color theme="1"/>
-        <sz val="11.0"/>
       </rPr>
       <t xml:space="preserve">Veuillez déclarer votre incident à la CNIL ici : 
 </t>
     </r>
     <r>
       <rPr>
+        <u val="single"/>
+        <sz val="11"/>
+        <color rgb="FF1155CC"/>
         <rFont val="Arial"/>
-        <color rgb="FF1155CC"/>
-        <sz val="11.0"/>
-        <u/>
       </rPr>
       <t>https://www.cnil.fr/fr/services-en-ligne/notifier-une-violation-de-donnees-personnelles</t>
     </r>
   </si>
   <si>
-    <t>Accès restreint, copie papier et numérique séparée en accès dégradé</t>
+    <t xml:space="preserve">Accès restreint, copie papier et numérique séparée en accès dégradé</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="10">
     <font>
-      <sz val="10.0"/>
-      <color rgb="FF000000"/>
+      <sz val="10.000000"/>
+      <color indexed="64"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -401,12 +406,12 @@
     </font>
     <font/>
     <font>
-      <sz val="12.0"/>
+      <sz val="12.000000"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
@@ -421,20 +426,20 @@
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="11.000000"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="16.0"/>
-      <color rgb="FFFF0000"/>
+      <sz val="16.000000"/>
+      <color indexed="2"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -443,12 +448,12 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <fgColor indexed="65"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
@@ -476,28 +481,40 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
-    <border/>
+  <borders count="18">
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
     <border>
       <left style="thin">
         <color rgb="FF999999"/>
       </left>
+      <right style="none"/>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
+      <diagonal style="none"/>
     </border>
     <border>
+      <left style="none"/>
+      <right style="none"/>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
+      <diagonal style="none"/>
     </border>
     <border>
+      <left style="none"/>
       <right style="thin">
         <color rgb="FF999999"/>
       </right>
@@ -507,27 +524,38 @@
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF999999"/>
       </left>
+      <right style="none"/>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
+      <left style="none"/>
+      <right style="none"/>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
+      <left style="none"/>
       <right style="thin">
         <color rgb="FF999999"/>
       </right>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="medium">
@@ -542,6 +570,7 @@
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -556,6 +585,7 @@
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -570,6 +600,7 @@
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -581,6 +612,8 @@
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -595,6 +628,7 @@
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
@@ -603,9 +637,57 @@
       <right style="thin">
         <color rgb="FF999999"/>
       </right>
+      <top style="none"/>
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF999999"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin">
@@ -614,105 +696,121 @@
       <right style="thin">
         <color rgb="FF999999"/>
       </right>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="36">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf fontId="1" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf fontId="1" fillId="2" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf fontId="2" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="1" fillId="2" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="4" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf fontId="3" fillId="2" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="5" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf fontId="2" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="2" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="4" fillId="3" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="8" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf fontId="4" fillId="3" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="9" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf fontId="4" fillId="3" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="10" fillId="4" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf fontId="4" fillId="4" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf fontId="4" fillId="0" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf fontId="4" fillId="0" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="12" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="11" fillId="5" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf fontId="2" fillId="0" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="6" fillId="2" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf fontId="7" fillId="5" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="7" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="10" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf fontId="4" fillId="6" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf fontId="4" fillId="0" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="11" fillId="2" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="11" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf fontId="4" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="4" fillId="2" borderId="13" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="6" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf fontId="4" fillId="2" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="13" fillId="0" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="11" fillId="6" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf fontId="4" fillId="2" borderId="15" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="16" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="17" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="4" fillId="6" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="11" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf fontId="8" fillId="0" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf fontId="9" fillId="5" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
@@ -720,19 +818,21 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="2152650" cy="628650"/>
+    <xdr:ext cx="2152650" cy="628649"/>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="0" name="image1.png"/>
-        <xdr:cNvPicPr preferRelativeResize="0"/>
+        <xdr:cNvPicPr/>
       </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
       </xdr:blipFill>
-      <xdr:spPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
@@ -744,12 +844,291 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -806,7 +1185,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -832,7 +1211,7 @@
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -909,7 +1288,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -939,24 +1318,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
+  <sheetFormatPr defaultColWidth="12.630000000000001" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="28.25"/>
-    <col customWidth="1" min="2" max="2" width="32.38"/>
-    <col customWidth="1" min="3" max="3" width="25.88"/>
-    <col customWidth="1" min="4" max="4" width="38.63"/>
+    <col customWidth="1" min="2" max="2" width="32.380000000000003"/>
+    <col customWidth="1" min="3" max="3" width="25.879999999999999"/>
+    <col customWidth="1" min="4" max="4" width="38.630000000000003"/>
     <col customWidth="1" min="5" max="5" width="29.25"/>
-    <col customWidth="1" min="6" max="6" width="28.0"/>
-    <col customWidth="1" min="7" max="7" width="17.13"/>
-    <col customWidth="1" min="8" max="8" width="84.0"/>
+    <col customWidth="1" min="6" max="6" width="28"/>
+    <col customWidth="1" min="7" max="7" width="17.129999999999999"/>
+    <col customWidth="1" min="8" max="8" width="84"/>
   </cols>
   <sheetData>
     <row r="1" ht="80.25" customHeight="1">
@@ -1111,7 +1492,7 @@
       <c r="Y5" s="15"/>
       <c r="Z5" s="15"/>
     </row>
-    <row r="6" ht="42.0" customHeight="1">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="17"/>
     </row>
     <row r="7" ht="35.25" customHeight="1">
@@ -1290,13 +1671,13 @@
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="A13" s="25"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="27"/>
     </row>
     <row r="14" ht="34.5" customHeight="1">
       <c r="A14" s="20" t="s">
@@ -1359,32 +1740,32 @@
       <c r="Z15" s="15"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="26"/>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
+      <c r="A16" s="28"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
-      <c r="I16" s="29"/>
-      <c r="J16" s="29"/>
-      <c r="K16" s="29"/>
-      <c r="L16" s="29"/>
-      <c r="M16" s="29"/>
-      <c r="N16" s="29"/>
-      <c r="O16" s="29"/>
-      <c r="P16" s="29"/>
-      <c r="Q16" s="29"/>
-      <c r="R16" s="29"/>
-      <c r="S16" s="29"/>
-      <c r="T16" s="29"/>
-      <c r="U16" s="29"/>
-      <c r="V16" s="29"/>
-      <c r="W16" s="29"/>
-      <c r="X16" s="29"/>
-      <c r="Y16" s="29"/>
-      <c r="Z16" s="29"/>
+      <c r="H16" s="29"/>
+      <c r="I16" s="30"/>
+      <c r="J16" s="30"/>
+      <c r="K16" s="30"/>
+      <c r="L16" s="30"/>
+      <c r="M16" s="30"/>
+      <c r="N16" s="30"/>
+      <c r="O16" s="30"/>
+      <c r="P16" s="30"/>
+      <c r="Q16" s="30"/>
+      <c r="R16" s="30"/>
+      <c r="S16" s="30"/>
+      <c r="T16" s="30"/>
+      <c r="U16" s="30"/>
+      <c r="V16" s="30"/>
+      <c r="W16" s="30"/>
+      <c r="X16" s="30"/>
+      <c r="Y16" s="30"/>
+      <c r="Z16" s="30"/>
     </row>
     <row r="17" ht="34.5" customHeight="1">
       <c r="A17" s="20" t="s">
@@ -1447,32 +1828,32 @@
       <c r="Z18" s="15"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="26"/>
-      <c r="B19" s="27"/>
-      <c r="C19" s="27"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
+      <c r="A19" s="28"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
       <c r="G19" s="28"/>
-      <c r="H19" s="28"/>
-      <c r="I19" s="29"/>
-      <c r="J19" s="29"/>
-      <c r="K19" s="29"/>
-      <c r="L19" s="29"/>
-      <c r="M19" s="29"/>
-      <c r="N19" s="29"/>
-      <c r="O19" s="29"/>
-      <c r="P19" s="29"/>
-      <c r="Q19" s="29"/>
-      <c r="R19" s="29"/>
-      <c r="S19" s="29"/>
-      <c r="T19" s="29"/>
-      <c r="U19" s="29"/>
-      <c r="V19" s="29"/>
-      <c r="W19" s="29"/>
-      <c r="X19" s="29"/>
-      <c r="Y19" s="29"/>
-      <c r="Z19" s="29"/>
+      <c r="H19" s="29"/>
+      <c r="I19" s="30"/>
+      <c r="J19" s="30"/>
+      <c r="K19" s="30"/>
+      <c r="L19" s="30"/>
+      <c r="M19" s="30"/>
+      <c r="N19" s="30"/>
+      <c r="O19" s="30"/>
+      <c r="P19" s="30"/>
+      <c r="Q19" s="30"/>
+      <c r="R19" s="30"/>
+      <c r="S19" s="30"/>
+      <c r="T19" s="30"/>
+      <c r="U19" s="30"/>
+      <c r="V19" s="30"/>
+      <c r="W19" s="30"/>
+      <c r="X19" s="30"/>
+      <c r="Y19" s="30"/>
+      <c r="Z19" s="30"/>
     </row>
     <row r="20" ht="34.5" customHeight="1">
       <c r="A20" s="20" t="s">
@@ -1535,32 +1916,32 @@
       <c r="Z21" s="15"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="26"/>
-      <c r="B22" s="27"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
+      <c r="A22" s="28"/>
+      <c r="B22" s="28"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
       <c r="G22" s="28"/>
-      <c r="H22" s="28"/>
-      <c r="I22" s="29"/>
-      <c r="J22" s="29"/>
-      <c r="K22" s="29"/>
-      <c r="L22" s="29"/>
-      <c r="M22" s="29"/>
-      <c r="N22" s="29"/>
-      <c r="O22" s="29"/>
-      <c r="P22" s="29"/>
-      <c r="Q22" s="29"/>
-      <c r="R22" s="29"/>
-      <c r="S22" s="29"/>
-      <c r="T22" s="29"/>
-      <c r="U22" s="29"/>
-      <c r="V22" s="29"/>
-      <c r="W22" s="29"/>
-      <c r="X22" s="29"/>
-      <c r="Y22" s="29"/>
-      <c r="Z22" s="29"/>
+      <c r="H22" s="29"/>
+      <c r="I22" s="30"/>
+      <c r="J22" s="30"/>
+      <c r="K22" s="30"/>
+      <c r="L22" s="30"/>
+      <c r="M22" s="30"/>
+      <c r="N22" s="30"/>
+      <c r="O22" s="30"/>
+      <c r="P22" s="30"/>
+      <c r="Q22" s="30"/>
+      <c r="R22" s="30"/>
+      <c r="S22" s="30"/>
+      <c r="T22" s="30"/>
+      <c r="U22" s="30"/>
+      <c r="V22" s="30"/>
+      <c r="W22" s="30"/>
+      <c r="X22" s="30"/>
+      <c r="Y22" s="30"/>
+      <c r="Z22" s="30"/>
     </row>
     <row r="23" ht="34.5" customHeight="1">
       <c r="A23" s="20" t="s">
@@ -1623,32 +2004,32 @@
       <c r="Z24" s="15"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="26"/>
-      <c r="B25" s="27"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="27"/>
+      <c r="A25" s="28"/>
+      <c r="B25" s="28"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="28"/>
+      <c r="E25" s="28"/>
+      <c r="F25" s="28"/>
       <c r="G25" s="28"/>
-      <c r="H25" s="28"/>
-      <c r="I25" s="29"/>
-      <c r="J25" s="29"/>
-      <c r="K25" s="29"/>
-      <c r="L25" s="29"/>
-      <c r="M25" s="29"/>
-      <c r="N25" s="29"/>
-      <c r="O25" s="29"/>
-      <c r="P25" s="29"/>
-      <c r="Q25" s="29"/>
-      <c r="R25" s="29"/>
-      <c r="S25" s="29"/>
-      <c r="T25" s="29"/>
-      <c r="U25" s="29"/>
-      <c r="V25" s="29"/>
-      <c r="W25" s="29"/>
-      <c r="X25" s="29"/>
-      <c r="Y25" s="29"/>
-      <c r="Z25" s="29"/>
+      <c r="H25" s="29"/>
+      <c r="I25" s="30"/>
+      <c r="J25" s="30"/>
+      <c r="K25" s="30"/>
+      <c r="L25" s="30"/>
+      <c r="M25" s="30"/>
+      <c r="N25" s="30"/>
+      <c r="O25" s="30"/>
+      <c r="P25" s="30"/>
+      <c r="Q25" s="30"/>
+      <c r="R25" s="30"/>
+      <c r="S25" s="30"/>
+      <c r="T25" s="30"/>
+      <c r="U25" s="30"/>
+      <c r="V25" s="30"/>
+      <c r="W25" s="30"/>
+      <c r="X25" s="30"/>
+      <c r="Y25" s="30"/>
+      <c r="Z25" s="30"/>
     </row>
     <row r="26" ht="34.5" customHeight="1">
       <c r="A26" s="20" t="s">
@@ -1711,32 +2092,32 @@
       <c r="Z27" s="15"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="26"/>
-      <c r="B28" s="27"/>
-      <c r="C28" s="27"/>
-      <c r="D28" s="27"/>
-      <c r="E28" s="27"/>
-      <c r="F28" s="27"/>
+      <c r="A28" s="28"/>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+      <c r="F28" s="28"/>
       <c r="G28" s="28"/>
-      <c r="H28" s="28"/>
-      <c r="I28" s="29"/>
-      <c r="J28" s="29"/>
-      <c r="K28" s="29"/>
-      <c r="L28" s="29"/>
-      <c r="M28" s="29"/>
-      <c r="N28" s="29"/>
-      <c r="O28" s="29"/>
-      <c r="P28" s="29"/>
-      <c r="Q28" s="29"/>
-      <c r="R28" s="29"/>
-      <c r="S28" s="29"/>
-      <c r="T28" s="29"/>
-      <c r="U28" s="29"/>
-      <c r="V28" s="29"/>
-      <c r="W28" s="29"/>
-      <c r="X28" s="29"/>
-      <c r="Y28" s="29"/>
-      <c r="Z28" s="29"/>
+      <c r="H28" s="29"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="30"/>
+      <c r="O28" s="30"/>
+      <c r="P28" s="30"/>
+      <c r="Q28" s="30"/>
+      <c r="R28" s="30"/>
+      <c r="S28" s="30"/>
+      <c r="T28" s="30"/>
+      <c r="U28" s="30"/>
+      <c r="V28" s="30"/>
+      <c r="W28" s="30"/>
+      <c r="X28" s="30"/>
+      <c r="Y28" s="30"/>
+      <c r="Z28" s="30"/>
     </row>
     <row r="29" ht="34.5" customHeight="1">
       <c r="A29" s="20" t="s">
@@ -1799,32 +2180,32 @@
       <c r="Z30" s="15"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="26"/>
-      <c r="B31" s="27"/>
-      <c r="C31" s="27"/>
-      <c r="D31" s="27"/>
-      <c r="E31" s="27"/>
-      <c r="F31" s="27"/>
+      <c r="A31" s="28"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
       <c r="G31" s="28"/>
-      <c r="H31" s="28"/>
-      <c r="I31" s="29"/>
-      <c r="J31" s="29"/>
-      <c r="K31" s="29"/>
-      <c r="L31" s="29"/>
-      <c r="M31" s="29"/>
-      <c r="N31" s="29"/>
-      <c r="O31" s="29"/>
-      <c r="P31" s="29"/>
-      <c r="Q31" s="29"/>
-      <c r="R31" s="29"/>
-      <c r="S31" s="29"/>
-      <c r="T31" s="29"/>
-      <c r="U31" s="29"/>
-      <c r="V31" s="29"/>
-      <c r="W31" s="29"/>
-      <c r="X31" s="29"/>
-      <c r="Y31" s="29"/>
-      <c r="Z31" s="29"/>
+      <c r="H31" s="29"/>
+      <c r="I31" s="30"/>
+      <c r="J31" s="30"/>
+      <c r="K31" s="30"/>
+      <c r="L31" s="30"/>
+      <c r="M31" s="30"/>
+      <c r="N31" s="30"/>
+      <c r="O31" s="30"/>
+      <c r="P31" s="30"/>
+      <c r="Q31" s="30"/>
+      <c r="R31" s="30"/>
+      <c r="S31" s="30"/>
+      <c r="T31" s="30"/>
+      <c r="U31" s="30"/>
+      <c r="V31" s="30"/>
+      <c r="W31" s="30"/>
+      <c r="X31" s="30"/>
+      <c r="Y31" s="30"/>
+      <c r="Z31" s="30"/>
     </row>
     <row r="32" ht="34.5" customHeight="1">
       <c r="A32" s="20" t="s">
@@ -1887,32 +2268,32 @@
       <c r="Z33" s="15"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="26"/>
-      <c r="B34" s="27"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
+      <c r="A34" s="28"/>
+      <c r="B34" s="28"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28"/>
       <c r="G34" s="28"/>
-      <c r="H34" s="28"/>
-      <c r="I34" s="29"/>
-      <c r="J34" s="29"/>
-      <c r="K34" s="29"/>
-      <c r="L34" s="29"/>
-      <c r="M34" s="29"/>
-      <c r="N34" s="29"/>
-      <c r="O34" s="29"/>
-      <c r="P34" s="29"/>
-      <c r="Q34" s="29"/>
-      <c r="R34" s="29"/>
-      <c r="S34" s="29"/>
-      <c r="T34" s="29"/>
-      <c r="U34" s="29"/>
-      <c r="V34" s="29"/>
-      <c r="W34" s="29"/>
-      <c r="X34" s="29"/>
-      <c r="Y34" s="29"/>
-      <c r="Z34" s="29"/>
+      <c r="H34" s="29"/>
+      <c r="I34" s="30"/>
+      <c r="J34" s="30"/>
+      <c r="K34" s="30"/>
+      <c r="L34" s="30"/>
+      <c r="M34" s="30"/>
+      <c r="N34" s="30"/>
+      <c r="O34" s="30"/>
+      <c r="P34" s="30"/>
+      <c r="Q34" s="30"/>
+      <c r="R34" s="30"/>
+      <c r="S34" s="30"/>
+      <c r="T34" s="30"/>
+      <c r="U34" s="30"/>
+      <c r="V34" s="30"/>
+      <c r="W34" s="30"/>
+      <c r="X34" s="30"/>
+      <c r="Y34" s="30"/>
+      <c r="Z34" s="30"/>
     </row>
     <row r="35" ht="34.5" customHeight="1">
       <c r="A35" s="20" t="s">
@@ -1975,32 +2356,32 @@
       <c r="Z36" s="15"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="26"/>
-      <c r="B37" s="27"/>
-      <c r="C37" s="27"/>
-      <c r="D37" s="27"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="27"/>
+      <c r="A37" s="28"/>
+      <c r="B37" s="28"/>
+      <c r="C37" s="28"/>
+      <c r="D37" s="28"/>
+      <c r="E37" s="28"/>
+      <c r="F37" s="28"/>
       <c r="G37" s="28"/>
-      <c r="H37" s="28"/>
-      <c r="I37" s="29"/>
-      <c r="J37" s="29"/>
-      <c r="K37" s="29"/>
-      <c r="L37" s="29"/>
-      <c r="M37" s="29"/>
-      <c r="N37" s="29"/>
-      <c r="O37" s="29"/>
-      <c r="P37" s="29"/>
-      <c r="Q37" s="29"/>
-      <c r="R37" s="29"/>
-      <c r="S37" s="29"/>
-      <c r="T37" s="29"/>
-      <c r="U37" s="29"/>
-      <c r="V37" s="29"/>
-      <c r="W37" s="29"/>
-      <c r="X37" s="29"/>
-      <c r="Y37" s="29"/>
-      <c r="Z37" s="29"/>
+      <c r="H37" s="29"/>
+      <c r="I37" s="30"/>
+      <c r="J37" s="30"/>
+      <c r="K37" s="30"/>
+      <c r="L37" s="30"/>
+      <c r="M37" s="30"/>
+      <c r="N37" s="30"/>
+      <c r="O37" s="30"/>
+      <c r="P37" s="30"/>
+      <c r="Q37" s="30"/>
+      <c r="R37" s="30"/>
+      <c r="S37" s="30"/>
+      <c r="T37" s="30"/>
+      <c r="U37" s="30"/>
+      <c r="V37" s="30"/>
+      <c r="W37" s="30"/>
+      <c r="X37" s="30"/>
+      <c r="Y37" s="30"/>
+      <c r="Z37" s="30"/>
     </row>
     <row r="38" ht="34.5" customHeight="1">
       <c r="A38" s="20" t="s">
@@ -2063,32 +2444,32 @@
       <c r="Z39" s="15"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="26"/>
-      <c r="B40" s="27"/>
-      <c r="C40" s="27"/>
-      <c r="D40" s="27"/>
-      <c r="E40" s="27"/>
-      <c r="F40" s="27"/>
+      <c r="A40" s="28"/>
+      <c r="B40" s="28"/>
+      <c r="C40" s="28"/>
+      <c r="D40" s="28"/>
+      <c r="E40" s="28"/>
+      <c r="F40" s="28"/>
       <c r="G40" s="28"/>
-      <c r="H40" s="28"/>
-      <c r="I40" s="29"/>
-      <c r="J40" s="29"/>
-      <c r="K40" s="29"/>
-      <c r="L40" s="29"/>
-      <c r="M40" s="29"/>
-      <c r="N40" s="29"/>
-      <c r="O40" s="29"/>
-      <c r="P40" s="29"/>
-      <c r="Q40" s="29"/>
-      <c r="R40" s="29"/>
-      <c r="S40" s="29"/>
-      <c r="T40" s="29"/>
-      <c r="U40" s="29"/>
-      <c r="V40" s="29"/>
-      <c r="W40" s="29"/>
-      <c r="X40" s="29"/>
-      <c r="Y40" s="29"/>
-      <c r="Z40" s="29"/>
+      <c r="H40" s="29"/>
+      <c r="I40" s="30"/>
+      <c r="J40" s="30"/>
+      <c r="K40" s="30"/>
+      <c r="L40" s="30"/>
+      <c r="M40" s="30"/>
+      <c r="N40" s="30"/>
+      <c r="O40" s="30"/>
+      <c r="P40" s="30"/>
+      <c r="Q40" s="30"/>
+      <c r="R40" s="30"/>
+      <c r="S40" s="30"/>
+      <c r="T40" s="30"/>
+      <c r="U40" s="30"/>
+      <c r="V40" s="30"/>
+      <c r="W40" s="30"/>
+      <c r="X40" s="30"/>
+      <c r="Y40" s="30"/>
+      <c r="Z40" s="30"/>
     </row>
     <row r="41" ht="40.5" customHeight="1">
       <c r="A41" s="20" t="s">
@@ -2226,13 +2607,13 @@
     </row>
     <row r="46" ht="17.25" customHeight="1">
       <c r="A46" s="25"/>
-      <c r="B46" s="25"/>
-      <c r="C46" s="25"/>
-      <c r="D46" s="25"/>
-      <c r="E46" s="25"/>
-      <c r="F46" s="25"/>
-      <c r="G46" s="25"/>
-      <c r="H46" s="25"/>
+      <c r="B46" s="26"/>
+      <c r="C46" s="26"/>
+      <c r="D46" s="26"/>
+      <c r="E46" s="26"/>
+      <c r="F46" s="26"/>
+      <c r="G46" s="26"/>
+      <c r="H46" s="27"/>
     </row>
     <row r="47" ht="33.75" customHeight="1">
       <c r="A47" s="20" t="s">
@@ -2617,7 +2998,7 @@
       <c r="Z62" s="15"/>
     </row>
     <row r="63" ht="33.75" customHeight="1">
-      <c r="A63" s="30"/>
+      <c r="A63" s="31"/>
       <c r="B63" s="13"/>
       <c r="C63" s="14"/>
       <c r="D63" s="14"/>
@@ -2715,7 +3096,7 @@
       <c r="Z66" s="15"/>
     </row>
     <row r="67" ht="33.75" customHeight="1">
-      <c r="A67" s="30"/>
+      <c r="A67" s="31"/>
       <c r="B67" s="13"/>
       <c r="C67" s="14"/>
       <c r="D67" s="14"/>
@@ -2851,7 +3232,7 @@
       <c r="H72" s="24"/>
     </row>
     <row r="73" ht="33.75" customHeight="1">
-      <c r="A73" s="31" t="s">
+      <c r="A73" s="32" t="s">
         <v>51</v>
       </c>
       <c r="B73" s="13"/>
@@ -2862,7 +3243,7 @@
       <c r="G73" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="H73" s="32" t="s">
+      <c r="H73" s="33" t="s">
         <v>52</v>
       </c>
       <c r="I73" s="15"/>
@@ -2885,821 +3266,821 @@
       <c r="Z73" s="15"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="G74" s="33"/>
+      <c r="G74" s="34"/>
       <c r="H74" s="15"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="G75" s="33"/>
+      <c r="G75" s="34"/>
       <c r="H75" s="15"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="G76" s="33"/>
+      <c r="G76" s="34"/>
       <c r="H76" s="15"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="G77" s="33"/>
+      <c r="G77" s="34"/>
       <c r="H77" s="15"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="34" t="s">
+      <c r="A78" s="35" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1"/>
     <row r="80" ht="15.75" hidden="1" customHeight="1">
-      <c r="G80" s="33"/>
+      <c r="G80" s="34"/>
       <c r="H80" s="15"/>
     </row>
     <row r="81" ht="15.75" hidden="1" customHeight="1">
-      <c r="G81" s="33"/>
+      <c r="G81" s="34"/>
       <c r="H81" s="15"/>
     </row>
     <row r="82" ht="15.75" hidden="1" customHeight="1">
-      <c r="G82" s="33"/>
+      <c r="G82" s="34"/>
       <c r="H82" s="15"/>
     </row>
     <row r="83" ht="15.75" hidden="1" customHeight="1">
-      <c r="G83" s="33"/>
+      <c r="G83" s="34"/>
       <c r="H83" s="15"/>
     </row>
     <row r="84" ht="15.75" hidden="1" customHeight="1">
-      <c r="G84" s="33"/>
+      <c r="G84" s="34"/>
       <c r="H84" s="15"/>
     </row>
     <row r="85" ht="15.75" hidden="1" customHeight="1">
-      <c r="G85" s="33"/>
+      <c r="G85" s="34"/>
       <c r="H85" s="15"/>
     </row>
     <row r="86" ht="15.75" hidden="1" customHeight="1">
-      <c r="G86" s="33"/>
+      <c r="G86" s="34"/>
       <c r="H86" s="15"/>
     </row>
     <row r="87" ht="15.75" hidden="1" customHeight="1">
-      <c r="G87" s="33"/>
+      <c r="G87" s="34"/>
       <c r="H87" s="15"/>
     </row>
     <row r="88" ht="15.75" hidden="1" customHeight="1">
-      <c r="G88" s="33"/>
+      <c r="G88" s="34"/>
       <c r="H88" s="15"/>
     </row>
     <row r="89" ht="15.75" hidden="1" customHeight="1">
-      <c r="G89" s="33"/>
+      <c r="G89" s="34"/>
       <c r="H89" s="15"/>
     </row>
     <row r="90" ht="15.75" hidden="1" customHeight="1">
-      <c r="G90" s="33"/>
+      <c r="G90" s="34"/>
       <c r="H90" s="15"/>
     </row>
     <row r="91" ht="15.75" hidden="1" customHeight="1">
-      <c r="G91" s="33"/>
+      <c r="G91" s="34"/>
       <c r="H91" s="15"/>
     </row>
     <row r="92" ht="15.75" hidden="1" customHeight="1">
-      <c r="G92" s="33"/>
+      <c r="G92" s="34"/>
       <c r="H92" s="15"/>
     </row>
     <row r="93" ht="15.75" hidden="1" customHeight="1">
-      <c r="G93" s="33"/>
+      <c r="G93" s="34"/>
       <c r="H93" s="15"/>
     </row>
     <row r="94" ht="15.75" hidden="1" customHeight="1">
-      <c r="G94" s="33"/>
+      <c r="G94" s="34"/>
       <c r="H94" s="15"/>
     </row>
     <row r="95" ht="15.75" hidden="1" customHeight="1">
-      <c r="G95" s="33"/>
+      <c r="G95" s="34"/>
       <c r="H95" s="15"/>
     </row>
     <row r="96" ht="15.75" hidden="1" customHeight="1">
-      <c r="G96" s="33"/>
+      <c r="G96" s="34"/>
       <c r="H96" s="15"/>
     </row>
     <row r="97" ht="15.75" hidden="1" customHeight="1">
-      <c r="G97" s="33"/>
+      <c r="G97" s="34"/>
       <c r="H97" s="15"/>
     </row>
     <row r="98" ht="15.75" hidden="1" customHeight="1">
-      <c r="G98" s="33"/>
+      <c r="G98" s="34"/>
       <c r="H98" s="15"/>
     </row>
     <row r="99" ht="15.75" hidden="1" customHeight="1">
-      <c r="G99" s="33"/>
+      <c r="G99" s="34"/>
       <c r="H99" s="15"/>
     </row>
     <row r="100" ht="15.75" hidden="1" customHeight="1">
-      <c r="G100" s="33"/>
+      <c r="G100" s="34"/>
       <c r="H100" s="15"/>
     </row>
     <row r="101" ht="15.75" hidden="1" customHeight="1">
-      <c r="G101" s="33"/>
+      <c r="G101" s="34"/>
       <c r="H101" s="15"/>
     </row>
     <row r="102" ht="15.75" hidden="1" customHeight="1">
-      <c r="G102" s="33"/>
+      <c r="G102" s="34"/>
       <c r="H102" s="15"/>
     </row>
     <row r="103" ht="15.75" hidden="1" customHeight="1">
-      <c r="G103" s="33"/>
+      <c r="G103" s="34"/>
       <c r="H103" s="15"/>
     </row>
     <row r="104" ht="15.75" hidden="1" customHeight="1">
-      <c r="G104" s="33"/>
+      <c r="G104" s="34"/>
       <c r="H104" s="15"/>
     </row>
     <row r="105" ht="15.75" hidden="1" customHeight="1">
-      <c r="G105" s="33"/>
+      <c r="G105" s="34"/>
       <c r="H105" s="15"/>
     </row>
     <row r="106" ht="15.75" hidden="1" customHeight="1">
-      <c r="G106" s="33"/>
+      <c r="G106" s="34"/>
       <c r="H106" s="15"/>
     </row>
     <row r="107" ht="15.75" hidden="1" customHeight="1">
-      <c r="G107" s="33"/>
+      <c r="G107" s="34"/>
       <c r="H107" s="15"/>
     </row>
     <row r="108" ht="15.75" hidden="1" customHeight="1">
-      <c r="G108" s="33"/>
+      <c r="G108" s="34"/>
       <c r="H108" s="15"/>
     </row>
     <row r="109" ht="15.75" hidden="1" customHeight="1">
-      <c r="G109" s="33"/>
+      <c r="G109" s="34"/>
       <c r="H109" s="15"/>
     </row>
     <row r="110" ht="15.75" hidden="1" customHeight="1">
-      <c r="G110" s="33"/>
+      <c r="G110" s="34"/>
       <c r="H110" s="15"/>
     </row>
     <row r="111" ht="15.75" hidden="1" customHeight="1">
-      <c r="G111" s="33"/>
+      <c r="G111" s="34"/>
       <c r="H111" s="15"/>
     </row>
     <row r="112" ht="15.75" hidden="1" customHeight="1">
-      <c r="G112" s="33"/>
+      <c r="G112" s="34"/>
       <c r="H112" s="15"/>
     </row>
     <row r="113" ht="15.75" hidden="1" customHeight="1">
-      <c r="G113" s="33"/>
+      <c r="G113" s="34"/>
       <c r="H113" s="15"/>
     </row>
     <row r="114" ht="15.75" hidden="1" customHeight="1">
-      <c r="G114" s="33"/>
+      <c r="G114" s="34"/>
       <c r="H114" s="15"/>
     </row>
     <row r="115" ht="15.75" hidden="1" customHeight="1">
-      <c r="G115" s="33"/>
+      <c r="G115" s="34"/>
       <c r="H115" s="15"/>
     </row>
     <row r="116" ht="15.75" hidden="1" customHeight="1">
-      <c r="G116" s="33"/>
+      <c r="G116" s="34"/>
       <c r="H116" s="15"/>
     </row>
     <row r="117" ht="15.75" hidden="1" customHeight="1">
-      <c r="G117" s="33"/>
+      <c r="G117" s="34"/>
       <c r="H117" s="15"/>
     </row>
     <row r="118" ht="15.75" hidden="1" customHeight="1">
-      <c r="G118" s="33"/>
+      <c r="G118" s="34"/>
       <c r="H118" s="15"/>
     </row>
     <row r="119" ht="15.75" hidden="1" customHeight="1">
-      <c r="G119" s="33"/>
+      <c r="G119" s="34"/>
       <c r="H119" s="15"/>
     </row>
     <row r="120" ht="15.75" hidden="1" customHeight="1">
-      <c r="G120" s="33"/>
+      <c r="G120" s="34"/>
       <c r="H120" s="15"/>
     </row>
     <row r="121" ht="15.75" hidden="1" customHeight="1">
-      <c r="G121" s="33"/>
+      <c r="G121" s="34"/>
       <c r="H121" s="15"/>
     </row>
     <row r="122" ht="15.75" hidden="1" customHeight="1">
-      <c r="G122" s="33"/>
+      <c r="G122" s="34"/>
       <c r="H122" s="15"/>
     </row>
     <row r="123" ht="15.75" hidden="1" customHeight="1">
-      <c r="G123" s="33"/>
+      <c r="G123" s="34"/>
       <c r="H123" s="15"/>
     </row>
     <row r="124" ht="15.75" hidden="1" customHeight="1">
-      <c r="G124" s="33"/>
+      <c r="G124" s="34"/>
       <c r="H124" s="15"/>
     </row>
     <row r="125" ht="15.75" hidden="1" customHeight="1">
-      <c r="G125" s="33"/>
+      <c r="G125" s="34"/>
       <c r="H125" s="15"/>
     </row>
     <row r="126" ht="15.75" hidden="1" customHeight="1">
-      <c r="G126" s="33"/>
+      <c r="G126" s="34"/>
       <c r="H126" s="15"/>
     </row>
     <row r="127" ht="15.75" hidden="1" customHeight="1">
-      <c r="G127" s="33"/>
+      <c r="G127" s="34"/>
       <c r="H127" s="15"/>
     </row>
     <row r="128" ht="15.75" hidden="1" customHeight="1">
-      <c r="G128" s="33"/>
+      <c r="G128" s="34"/>
       <c r="H128" s="15"/>
     </row>
     <row r="129" ht="15.75" hidden="1" customHeight="1">
-      <c r="G129" s="33"/>
+      <c r="G129" s="34"/>
       <c r="H129" s="15"/>
     </row>
     <row r="130" ht="15.75" hidden="1" customHeight="1">
-      <c r="G130" s="33"/>
+      <c r="G130" s="34"/>
       <c r="H130" s="15"/>
     </row>
     <row r="131" ht="15.75" hidden="1" customHeight="1">
-      <c r="G131" s="33"/>
+      <c r="G131" s="34"/>
       <c r="H131" s="15"/>
     </row>
     <row r="132" ht="15.75" hidden="1" customHeight="1">
-      <c r="G132" s="33"/>
+      <c r="G132" s="34"/>
       <c r="H132" s="15"/>
     </row>
     <row r="133" ht="15.75" hidden="1" customHeight="1">
-      <c r="G133" s="33"/>
+      <c r="G133" s="34"/>
       <c r="H133" s="15"/>
     </row>
     <row r="134" ht="15.75" hidden="1" customHeight="1">
-      <c r="G134" s="33"/>
+      <c r="G134" s="34"/>
       <c r="H134" s="15"/>
     </row>
     <row r="135" ht="15.75" hidden="1" customHeight="1">
-      <c r="G135" s="33"/>
+      <c r="G135" s="34"/>
       <c r="H135" s="15"/>
     </row>
     <row r="136" ht="15.75" hidden="1" customHeight="1">
-      <c r="G136" s="33"/>
+      <c r="G136" s="34"/>
       <c r="H136" s="15"/>
     </row>
     <row r="137" ht="15.75" hidden="1" customHeight="1">
-      <c r="G137" s="33"/>
+      <c r="G137" s="34"/>
       <c r="H137" s="15"/>
     </row>
     <row r="138" ht="15.75" hidden="1" customHeight="1">
-      <c r="G138" s="33"/>
+      <c r="G138" s="34"/>
       <c r="H138" s="15"/>
     </row>
     <row r="139" ht="15.75" hidden="1" customHeight="1">
-      <c r="G139" s="33"/>
+      <c r="G139" s="34"/>
       <c r="H139" s="15"/>
     </row>
     <row r="140" ht="15.75" hidden="1" customHeight="1">
-      <c r="G140" s="33"/>
+      <c r="G140" s="34"/>
       <c r="H140" s="15"/>
     </row>
     <row r="141" ht="15.75" hidden="1" customHeight="1">
-      <c r="G141" s="33"/>
+      <c r="G141" s="34"/>
       <c r="H141" s="15"/>
     </row>
     <row r="142" ht="15.75" hidden="1" customHeight="1">
-      <c r="G142" s="33"/>
+      <c r="G142" s="34"/>
       <c r="H142" s="15"/>
     </row>
     <row r="143" ht="15.75" hidden="1" customHeight="1">
-      <c r="G143" s="33"/>
+      <c r="G143" s="34"/>
       <c r="H143" s="15"/>
     </row>
     <row r="144" ht="15.75" hidden="1" customHeight="1">
-      <c r="G144" s="33"/>
+      <c r="G144" s="34"/>
       <c r="H144" s="15"/>
     </row>
     <row r="145" ht="15.75" hidden="1" customHeight="1">
-      <c r="G145" s="33"/>
+      <c r="G145" s="34"/>
       <c r="H145" s="15"/>
     </row>
     <row r="146" ht="15.75" hidden="1" customHeight="1">
-      <c r="G146" s="33"/>
+      <c r="G146" s="34"/>
       <c r="H146" s="15"/>
     </row>
     <row r="147" ht="15.75" hidden="1" customHeight="1">
-      <c r="G147" s="33"/>
+      <c r="G147" s="34"/>
       <c r="H147" s="15"/>
     </row>
     <row r="148" ht="15.75" hidden="1" customHeight="1">
-      <c r="G148" s="33"/>
+      <c r="G148" s="34"/>
       <c r="H148" s="15"/>
     </row>
     <row r="149" ht="15.75" hidden="1" customHeight="1">
-      <c r="G149" s="33"/>
+      <c r="G149" s="34"/>
       <c r="H149" s="15"/>
     </row>
     <row r="150" ht="15.75" hidden="1" customHeight="1">
-      <c r="G150" s="33"/>
+      <c r="G150" s="34"/>
       <c r="H150" s="15"/>
     </row>
     <row r="151" ht="15.75" hidden="1" customHeight="1">
-      <c r="G151" s="33"/>
+      <c r="G151" s="34"/>
       <c r="H151" s="15"/>
     </row>
     <row r="152" ht="15.75" hidden="1" customHeight="1">
-      <c r="G152" s="33"/>
+      <c r="G152" s="34"/>
       <c r="H152" s="15"/>
     </row>
     <row r="153" ht="15.75" hidden="1" customHeight="1">
-      <c r="G153" s="33"/>
+      <c r="G153" s="34"/>
       <c r="H153" s="15"/>
     </row>
     <row r="154" ht="15.75" hidden="1" customHeight="1">
-      <c r="G154" s="33"/>
+      <c r="G154" s="34"/>
       <c r="H154" s="15"/>
     </row>
     <row r="155" ht="15.75" hidden="1" customHeight="1">
-      <c r="G155" s="33"/>
+      <c r="G155" s="34"/>
       <c r="H155" s="15"/>
     </row>
     <row r="156" ht="15.75" hidden="1" customHeight="1">
-      <c r="G156" s="33"/>
+      <c r="G156" s="34"/>
       <c r="H156" s="15"/>
     </row>
     <row r="157" ht="15.75" hidden="1" customHeight="1">
-      <c r="G157" s="33"/>
+      <c r="G157" s="34"/>
       <c r="H157" s="15"/>
     </row>
     <row r="158" ht="15.75" hidden="1" customHeight="1">
-      <c r="G158" s="33"/>
+      <c r="G158" s="34"/>
       <c r="H158" s="15"/>
     </row>
     <row r="159" ht="15.75" hidden="1" customHeight="1">
-      <c r="G159" s="33"/>
+      <c r="G159" s="34"/>
       <c r="H159" s="15"/>
     </row>
     <row r="160" ht="15.75" hidden="1" customHeight="1">
-      <c r="G160" s="33"/>
+      <c r="G160" s="34"/>
       <c r="H160" s="15"/>
     </row>
     <row r="161" ht="15.75" hidden="1" customHeight="1">
-      <c r="G161" s="33"/>
+      <c r="G161" s="34"/>
       <c r="H161" s="15"/>
     </row>
     <row r="162" ht="15.75" hidden="1" customHeight="1">
-      <c r="G162" s="33"/>
+      <c r="G162" s="34"/>
       <c r="H162" s="15"/>
     </row>
     <row r="163" ht="15.75" hidden="1" customHeight="1">
-      <c r="G163" s="33"/>
+      <c r="G163" s="34"/>
       <c r="H163" s="15"/>
     </row>
     <row r="164" ht="15.75" hidden="1" customHeight="1">
-      <c r="G164" s="33"/>
+      <c r="G164" s="34"/>
       <c r="H164" s="15"/>
     </row>
     <row r="165" ht="15.75" hidden="1" customHeight="1">
-      <c r="G165" s="33"/>
+      <c r="G165" s="34"/>
       <c r="H165" s="15"/>
     </row>
     <row r="166" ht="15.75" hidden="1" customHeight="1">
-      <c r="G166" s="33"/>
+      <c r="G166" s="34"/>
       <c r="H166" s="15"/>
     </row>
     <row r="167" ht="15.75" hidden="1" customHeight="1">
-      <c r="G167" s="33"/>
+      <c r="G167" s="34"/>
       <c r="H167" s="15"/>
     </row>
     <row r="168" ht="15.75" hidden="1" customHeight="1">
-      <c r="G168" s="33"/>
+      <c r="G168" s="34"/>
       <c r="H168" s="15"/>
     </row>
     <row r="169" ht="15.75" hidden="1" customHeight="1">
-      <c r="G169" s="33"/>
+      <c r="G169" s="34"/>
       <c r="H169" s="15"/>
     </row>
     <row r="170" ht="15.75" hidden="1" customHeight="1">
-      <c r="G170" s="33"/>
+      <c r="G170" s="34"/>
       <c r="H170" s="15"/>
     </row>
     <row r="171" ht="15.75" hidden="1" customHeight="1">
-      <c r="G171" s="33"/>
+      <c r="G171" s="34"/>
       <c r="H171" s="15"/>
     </row>
     <row r="172" ht="15.75" hidden="1" customHeight="1">
-      <c r="G172" s="33"/>
+      <c r="G172" s="34"/>
       <c r="H172" s="15"/>
     </row>
     <row r="173" ht="15.75" hidden="1" customHeight="1">
-      <c r="G173" s="33"/>
+      <c r="G173" s="34"/>
       <c r="H173" s="15"/>
     </row>
     <row r="174" ht="15.75" hidden="1" customHeight="1">
-      <c r="G174" s="33"/>
+      <c r="G174" s="34"/>
       <c r="H174" s="15"/>
     </row>
     <row r="175" ht="15.75" hidden="1" customHeight="1">
-      <c r="G175" s="33"/>
+      <c r="G175" s="34"/>
       <c r="H175" s="15"/>
     </row>
     <row r="176" ht="15.75" hidden="1" customHeight="1">
-      <c r="G176" s="33"/>
+      <c r="G176" s="34"/>
       <c r="H176" s="15"/>
     </row>
     <row r="177" ht="15.75" hidden="1" customHeight="1">
-      <c r="G177" s="33"/>
+      <c r="G177" s="34"/>
       <c r="H177" s="15"/>
     </row>
     <row r="178" ht="15.75" hidden="1" customHeight="1">
-      <c r="G178" s="33"/>
+      <c r="G178" s="34"/>
       <c r="H178" s="15"/>
     </row>
     <row r="179" ht="15.75" hidden="1" customHeight="1">
-      <c r="G179" s="33"/>
+      <c r="G179" s="34"/>
       <c r="H179" s="15"/>
     </row>
     <row r="180" ht="15.75" hidden="1" customHeight="1">
-      <c r="G180" s="33"/>
+      <c r="G180" s="34"/>
       <c r="H180" s="15"/>
     </row>
     <row r="181" ht="15.75" hidden="1" customHeight="1">
-      <c r="G181" s="33"/>
+      <c r="G181" s="34"/>
       <c r="H181" s="15"/>
     </row>
     <row r="182" ht="15.75" hidden="1" customHeight="1">
-      <c r="G182" s="33"/>
+      <c r="G182" s="34"/>
       <c r="H182" s="15"/>
     </row>
     <row r="183" ht="15.75" hidden="1" customHeight="1">
-      <c r="G183" s="33"/>
+      <c r="G183" s="34"/>
       <c r="H183" s="15"/>
     </row>
     <row r="184" ht="15.75" hidden="1" customHeight="1">
-      <c r="G184" s="33"/>
+      <c r="G184" s="34"/>
       <c r="H184" s="15"/>
     </row>
     <row r="185" ht="15.75" hidden="1" customHeight="1">
-      <c r="G185" s="33"/>
+      <c r="G185" s="34"/>
       <c r="H185" s="15"/>
     </row>
     <row r="186" ht="15.75" hidden="1" customHeight="1">
-      <c r="G186" s="33"/>
+      <c r="G186" s="34"/>
       <c r="H186" s="15"/>
     </row>
     <row r="187" ht="15.75" hidden="1" customHeight="1">
-      <c r="G187" s="33"/>
+      <c r="G187" s="34"/>
       <c r="H187" s="15"/>
     </row>
     <row r="188" ht="15.75" hidden="1" customHeight="1">
-      <c r="G188" s="33"/>
+      <c r="G188" s="34"/>
       <c r="H188" s="15"/>
     </row>
     <row r="189" ht="15.75" hidden="1" customHeight="1">
-      <c r="G189" s="33"/>
+      <c r="G189" s="34"/>
       <c r="H189" s="15"/>
     </row>
     <row r="190" ht="15.75" hidden="1" customHeight="1">
-      <c r="G190" s="33"/>
+      <c r="G190" s="34"/>
       <c r="H190" s="15"/>
     </row>
     <row r="191" ht="15.75" hidden="1" customHeight="1">
-      <c r="G191" s="33"/>
+      <c r="G191" s="34"/>
       <c r="H191" s="15"/>
     </row>
     <row r="192" ht="15.75" hidden="1" customHeight="1">
-      <c r="G192" s="33"/>
+      <c r="G192" s="34"/>
       <c r="H192" s="15"/>
     </row>
     <row r="193" ht="15.75" hidden="1" customHeight="1">
-      <c r="G193" s="33"/>
+      <c r="G193" s="34"/>
       <c r="H193" s="15"/>
     </row>
     <row r="194" ht="15.75" hidden="1" customHeight="1">
-      <c r="G194" s="33"/>
+      <c r="G194" s="34"/>
       <c r="H194" s="15"/>
     </row>
     <row r="195" ht="15.75" hidden="1" customHeight="1">
-      <c r="G195" s="33"/>
+      <c r="G195" s="34"/>
       <c r="H195" s="15"/>
     </row>
     <row r="196" ht="15.75" hidden="1" customHeight="1">
-      <c r="G196" s="33"/>
+      <c r="G196" s="34"/>
       <c r="H196" s="15"/>
     </row>
     <row r="197" ht="15.75" hidden="1" customHeight="1">
-      <c r="G197" s="33"/>
+      <c r="G197" s="34"/>
       <c r="H197" s="15"/>
     </row>
     <row r="198" ht="15.75" hidden="1" customHeight="1">
-      <c r="G198" s="33"/>
+      <c r="G198" s="34"/>
       <c r="H198" s="15"/>
     </row>
     <row r="199" ht="15.75" hidden="1" customHeight="1">
-      <c r="G199" s="33"/>
+      <c r="G199" s="34"/>
       <c r="H199" s="15"/>
     </row>
     <row r="200" ht="15.75" hidden="1" customHeight="1">
-      <c r="G200" s="33"/>
+      <c r="G200" s="34"/>
       <c r="H200" s="15"/>
     </row>
     <row r="201" ht="15.75" hidden="1" customHeight="1">
-      <c r="G201" s="33"/>
+      <c r="G201" s="34"/>
       <c r="H201" s="15"/>
     </row>
     <row r="202" ht="15.75" hidden="1" customHeight="1">
-      <c r="G202" s="33"/>
+      <c r="G202" s="34"/>
       <c r="H202" s="15"/>
     </row>
     <row r="203" ht="15.75" hidden="1" customHeight="1">
-      <c r="G203" s="33"/>
+      <c r="G203" s="34"/>
       <c r="H203" s="15"/>
     </row>
     <row r="204" ht="15.75" hidden="1" customHeight="1">
-      <c r="G204" s="33"/>
+      <c r="G204" s="34"/>
       <c r="H204" s="15"/>
     </row>
     <row r="205" ht="15.75" hidden="1" customHeight="1">
-      <c r="G205" s="33"/>
+      <c r="G205" s="34"/>
       <c r="H205" s="15"/>
     </row>
     <row r="206" ht="15.75" hidden="1" customHeight="1">
-      <c r="G206" s="33"/>
+      <c r="G206" s="34"/>
       <c r="H206" s="15"/>
     </row>
     <row r="207" ht="15.75" hidden="1" customHeight="1">
-      <c r="G207" s="33"/>
+      <c r="G207" s="34"/>
       <c r="H207" s="15"/>
     </row>
     <row r="208" ht="15.75" hidden="1" customHeight="1">
-      <c r="G208" s="33"/>
+      <c r="G208" s="34"/>
       <c r="H208" s="15"/>
     </row>
     <row r="209" ht="15.75" hidden="1" customHeight="1">
-      <c r="G209" s="33"/>
+      <c r="G209" s="34"/>
       <c r="H209" s="15"/>
     </row>
     <row r="210" ht="15.75" hidden="1" customHeight="1">
-      <c r="G210" s="33"/>
+      <c r="G210" s="34"/>
       <c r="H210" s="15"/>
     </row>
     <row r="211" ht="15.75" hidden="1" customHeight="1">
-      <c r="G211" s="33"/>
+      <c r="G211" s="34"/>
       <c r="H211" s="15"/>
     </row>
     <row r="212" ht="15.75" hidden="1" customHeight="1">
-      <c r="G212" s="33"/>
+      <c r="G212" s="34"/>
       <c r="H212" s="15"/>
     </row>
     <row r="213" ht="15.75" hidden="1" customHeight="1">
-      <c r="G213" s="33"/>
+      <c r="G213" s="34"/>
       <c r="H213" s="15"/>
     </row>
     <row r="214" ht="15.75" hidden="1" customHeight="1">
-      <c r="G214" s="33"/>
+      <c r="G214" s="34"/>
       <c r="H214" s="15"/>
     </row>
     <row r="215" ht="15.75" hidden="1" customHeight="1">
-      <c r="G215" s="33"/>
+      <c r="G215" s="34"/>
       <c r="H215" s="15"/>
     </row>
     <row r="216" ht="15.75" hidden="1" customHeight="1">
-      <c r="G216" s="33"/>
+      <c r="G216" s="34"/>
       <c r="H216" s="15"/>
     </row>
     <row r="217" ht="15.75" hidden="1" customHeight="1">
-      <c r="G217" s="33"/>
+      <c r="G217" s="34"/>
       <c r="H217" s="15"/>
     </row>
     <row r="218" ht="15.75" hidden="1" customHeight="1">
-      <c r="G218" s="33"/>
+      <c r="G218" s="34"/>
       <c r="H218" s="15"/>
     </row>
     <row r="219" ht="15.75" hidden="1" customHeight="1">
-      <c r="G219" s="33"/>
+      <c r="G219" s="34"/>
       <c r="H219" s="15"/>
     </row>
     <row r="220" ht="15.75" hidden="1" customHeight="1">
-      <c r="G220" s="33"/>
+      <c r="G220" s="34"/>
       <c r="H220" s="15"/>
     </row>
     <row r="221" ht="15.75" hidden="1" customHeight="1">
-      <c r="G221" s="33"/>
+      <c r="G221" s="34"/>
       <c r="H221" s="15"/>
     </row>
     <row r="222" ht="15.75" hidden="1" customHeight="1">
-      <c r="G222" s="33"/>
+      <c r="G222" s="34"/>
       <c r="H222" s="15"/>
     </row>
     <row r="223" ht="15.75" hidden="1" customHeight="1">
-      <c r="G223" s="33"/>
+      <c r="G223" s="34"/>
       <c r="H223" s="15"/>
     </row>
     <row r="224" ht="15.75" hidden="1" customHeight="1">
-      <c r="G224" s="33"/>
+      <c r="G224" s="34"/>
       <c r="H224" s="15"/>
     </row>
     <row r="225" ht="15.75" hidden="1" customHeight="1">
-      <c r="G225" s="33"/>
+      <c r="G225" s="34"/>
       <c r="H225" s="15"/>
     </row>
     <row r="226" ht="15.75" hidden="1" customHeight="1">
-      <c r="G226" s="33"/>
+      <c r="G226" s="34"/>
       <c r="H226" s="15"/>
     </row>
     <row r="227" ht="15.75" hidden="1" customHeight="1">
-      <c r="G227" s="33"/>
+      <c r="G227" s="34"/>
       <c r="H227" s="15"/>
     </row>
     <row r="228" ht="15.75" hidden="1" customHeight="1">
-      <c r="G228" s="33"/>
+      <c r="G228" s="34"/>
       <c r="H228" s="15"/>
     </row>
     <row r="229" ht="15.75" hidden="1" customHeight="1">
-      <c r="G229" s="33"/>
+      <c r="G229" s="34"/>
       <c r="H229" s="15"/>
     </row>
     <row r="230" ht="15.75" hidden="1" customHeight="1">
-      <c r="G230" s="33"/>
+      <c r="G230" s="34"/>
       <c r="H230" s="15"/>
     </row>
     <row r="231" ht="15.75" hidden="1" customHeight="1">
-      <c r="G231" s="33"/>
+      <c r="G231" s="34"/>
       <c r="H231" s="15"/>
     </row>
     <row r="232" ht="15.75" hidden="1" customHeight="1">
-      <c r="G232" s="33"/>
+      <c r="G232" s="34"/>
       <c r="H232" s="15"/>
     </row>
     <row r="233" ht="15.75" hidden="1" customHeight="1">
-      <c r="G233" s="33"/>
+      <c r="G233" s="34"/>
       <c r="H233" s="15"/>
     </row>
     <row r="234" ht="15.75" hidden="1" customHeight="1">
-      <c r="G234" s="33"/>
+      <c r="G234" s="34"/>
       <c r="H234" s="15"/>
     </row>
     <row r="235" ht="15.75" hidden="1" customHeight="1">
-      <c r="G235" s="33"/>
+      <c r="G235" s="34"/>
       <c r="H235" s="15"/>
     </row>
     <row r="236" ht="15.75" hidden="1" customHeight="1">
-      <c r="G236" s="33"/>
+      <c r="G236" s="34"/>
       <c r="H236" s="15"/>
     </row>
     <row r="237" ht="15.75" hidden="1" customHeight="1">
-      <c r="G237" s="33"/>
+      <c r="G237" s="34"/>
       <c r="H237" s="15"/>
     </row>
     <row r="238" ht="15.75" hidden="1" customHeight="1">
-      <c r="G238" s="33"/>
+      <c r="G238" s="34"/>
       <c r="H238" s="15"/>
     </row>
     <row r="239" ht="15.75" hidden="1" customHeight="1">
-      <c r="G239" s="33"/>
+      <c r="G239" s="34"/>
       <c r="H239" s="15"/>
     </row>
     <row r="240" ht="15.75" hidden="1" customHeight="1">
-      <c r="G240" s="33"/>
+      <c r="G240" s="34"/>
       <c r="H240" s="15"/>
     </row>
     <row r="241" ht="15.75" hidden="1" customHeight="1">
-      <c r="G241" s="33"/>
+      <c r="G241" s="34"/>
       <c r="H241" s="15"/>
     </row>
     <row r="242" ht="15.75" hidden="1" customHeight="1">
-      <c r="G242" s="33"/>
+      <c r="G242" s="34"/>
       <c r="H242" s="15"/>
     </row>
     <row r="243" ht="15.75" hidden="1" customHeight="1">
-      <c r="G243" s="33"/>
+      <c r="G243" s="34"/>
       <c r="H243" s="15"/>
     </row>
     <row r="244" ht="15.75" hidden="1" customHeight="1">
-      <c r="G244" s="33"/>
+      <c r="G244" s="34"/>
       <c r="H244" s="15"/>
     </row>
     <row r="245" ht="15.75" hidden="1" customHeight="1">
-      <c r="G245" s="33"/>
+      <c r="G245" s="34"/>
       <c r="H245" s="15"/>
     </row>
     <row r="246" ht="15.75" hidden="1" customHeight="1">
-      <c r="G246" s="33"/>
+      <c r="G246" s="34"/>
       <c r="H246" s="15"/>
     </row>
     <row r="247" ht="15.75" hidden="1" customHeight="1">
-      <c r="G247" s="33"/>
+      <c r="G247" s="34"/>
       <c r="H247" s="15"/>
     </row>
     <row r="248" ht="15.75" hidden="1" customHeight="1">
-      <c r="G248" s="33"/>
+      <c r="G248" s="34"/>
       <c r="H248" s="15"/>
     </row>
     <row r="249" ht="15.75" hidden="1" customHeight="1">
-      <c r="G249" s="33"/>
+      <c r="G249" s="34"/>
       <c r="H249" s="15"/>
     </row>
     <row r="250" ht="15.75" hidden="1" customHeight="1">
-      <c r="G250" s="33"/>
+      <c r="G250" s="34"/>
       <c r="H250" s="15"/>
     </row>
     <row r="251" ht="15.75" hidden="1" customHeight="1">
-      <c r="G251" s="33"/>
+      <c r="G251" s="34"/>
       <c r="H251" s="15"/>
     </row>
     <row r="252" ht="15.75" hidden="1" customHeight="1">
-      <c r="G252" s="33"/>
+      <c r="G252" s="34"/>
       <c r="H252" s="15"/>
     </row>
     <row r="253" ht="15.75" hidden="1" customHeight="1">
-      <c r="G253" s="33"/>
+      <c r="G253" s="34"/>
       <c r="H253" s="15"/>
     </row>
     <row r="254" ht="15.75" hidden="1" customHeight="1">
-      <c r="G254" s="33"/>
+      <c r="G254" s="34"/>
       <c r="H254" s="15"/>
     </row>
     <row r="255" ht="15.75" hidden="1" customHeight="1">
-      <c r="G255" s="33"/>
+      <c r="G255" s="34"/>
       <c r="H255" s="15"/>
     </row>
     <row r="256" ht="15.75" hidden="1" customHeight="1">
-      <c r="G256" s="33"/>
+      <c r="G256" s="34"/>
       <c r="H256" s="15"/>
     </row>
     <row r="257" ht="15.75" hidden="1" customHeight="1">
-      <c r="G257" s="33"/>
+      <c r="G257" s="34"/>
       <c r="H257" s="15"/>
     </row>
     <row r="258" ht="15.75" hidden="1" customHeight="1">
-      <c r="G258" s="33"/>
+      <c r="G258" s="34"/>
       <c r="H258" s="15"/>
     </row>
     <row r="259" ht="15.75" hidden="1" customHeight="1">
-      <c r="G259" s="33"/>
+      <c r="G259" s="34"/>
       <c r="H259" s="15"/>
     </row>
     <row r="260" ht="15.75" hidden="1" customHeight="1">
-      <c r="G260" s="33"/>
+      <c r="G260" s="34"/>
       <c r="H260" s="15"/>
     </row>
     <row r="261" ht="15.75" hidden="1" customHeight="1">
-      <c r="G261" s="33"/>
+      <c r="G261" s="34"/>
       <c r="H261" s="15"/>
     </row>
     <row r="262" ht="15.75" hidden="1" customHeight="1">
-      <c r="G262" s="33"/>
+      <c r="G262" s="34"/>
       <c r="H262" s="15"/>
     </row>
     <row r="263" ht="15.75" hidden="1" customHeight="1">
-      <c r="G263" s="33"/>
+      <c r="G263" s="34"/>
       <c r="H263" s="15"/>
     </row>
     <row r="264" ht="15.75" hidden="1" customHeight="1">
-      <c r="G264" s="33"/>
+      <c r="G264" s="34"/>
       <c r="H264" s="15"/>
     </row>
     <row r="265" ht="15.75" hidden="1" customHeight="1">
-      <c r="G265" s="33"/>
+      <c r="G265" s="34"/>
       <c r="H265" s="15"/>
     </row>
     <row r="266" ht="15.75" hidden="1" customHeight="1">
-      <c r="G266" s="33"/>
+      <c r="G266" s="34"/>
       <c r="H266" s="15"/>
     </row>
     <row r="267" ht="15.75" hidden="1" customHeight="1">
-      <c r="G267" s="33"/>
+      <c r="G267" s="34"/>
       <c r="H267" s="15"/>
     </row>
     <row r="268" ht="15.75" hidden="1" customHeight="1">
-      <c r="G268" s="33"/>
+      <c r="G268" s="34"/>
       <c r="H268" s="15"/>
     </row>
     <row r="269" ht="15.75" hidden="1" customHeight="1">
-      <c r="G269" s="33"/>
+      <c r="G269" s="34"/>
       <c r="H269" s="15"/>
     </row>
     <row r="270" ht="15.75" hidden="1" customHeight="1">
-      <c r="G270" s="33"/>
+      <c r="G270" s="34"/>
       <c r="H270" s="15"/>
     </row>
     <row r="271" ht="15.75" hidden="1" customHeight="1">
-      <c r="G271" s="33"/>
+      <c r="G271" s="34"/>
       <c r="H271" s="15"/>
     </row>
     <row r="272" ht="15.75" hidden="1" customHeight="1">
-      <c r="G272" s="33"/>
+      <c r="G272" s="34"/>
       <c r="H272" s="15"/>
     </row>
     <row r="273" ht="15.75" hidden="1" customHeight="1">
-      <c r="G273" s="33"/>
+      <c r="G273" s="34"/>
       <c r="H273" s="15"/>
     </row>
     <row r="274" ht="15.75" hidden="1" customHeight="1">
-      <c r="G274" s="33"/>
+      <c r="G274" s="34"/>
       <c r="H274" s="15"/>
     </row>
     <row r="275" ht="15.75" hidden="1" customHeight="1">
-      <c r="G275" s="33"/>
+      <c r="G275" s="34"/>
       <c r="H275" s="15"/>
     </row>
     <row r="276" ht="15.75" hidden="1" customHeight="1">
-      <c r="G276" s="33"/>
+      <c r="G276" s="34"/>
       <c r="H276" s="15"/>
     </row>
     <row r="277" ht="15.75" hidden="1" customHeight="1">
-      <c r="G277" s="33"/>
+      <c r="G277" s="34"/>
       <c r="H277" s="15"/>
     </row>
     <row r="278" ht="15.75" hidden="1" customHeight="1">
-      <c r="G278" s="33"/>
+      <c r="G278" s="34"/>
       <c r="H278" s="15"/>
     </row>
     <row r="279" ht="15.75" customHeight="1">
@@ -5884,7 +6265,7 @@
       <c r="H1005" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="47">
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:A5"/>
@@ -5892,28 +6273,35 @@
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="A29:A30"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A34:H34"/>
     <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A37:H37"/>
     <mergeCell ref="A38:A39"/>
+    <mergeCell ref="A40:H40"/>
     <mergeCell ref="A41:A42"/>
     <mergeCell ref="A43:H43"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="A29:A30"/>
-    <mergeCell ref="A32:A33"/>
     <mergeCell ref="A44:A45"/>
+    <mergeCell ref="A46:H46"/>
     <mergeCell ref="A47:A48"/>
     <mergeCell ref="A49:H49"/>
     <mergeCell ref="A50:A51"/>
     <mergeCell ref="A52:H52"/>
     <mergeCell ref="A53:A54"/>
     <mergeCell ref="A55:H55"/>
-    <mergeCell ref="A69:H69"/>
-    <mergeCell ref="A72:H72"/>
-    <mergeCell ref="A78:H79"/>
-    <mergeCell ref="A70:A71"/>
     <mergeCell ref="A56:A57"/>
     <mergeCell ref="A58:H58"/>
     <mergeCell ref="A59:A60"/>
@@ -5921,10 +6309,18 @@
     <mergeCell ref="A62:A64"/>
     <mergeCell ref="A65:H65"/>
     <mergeCell ref="A66:A68"/>
+    <mergeCell ref="A69:H69"/>
+    <mergeCell ref="A70:A71"/>
+    <mergeCell ref="A72:H72"/>
+    <mergeCell ref="A78:H79"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="H73"/>
   </hyperlinks>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>